<commit_message>
Hooks updated for Taking Screenshot
</commit_message>
<xml_diff>
--- a/Excel/Account.xlsx
+++ b/Excel/Account.xlsx
@@ -14,16 +14,16 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
-    <t>Test New</t>
+    <t>SFQA Test</t>
   </si>
   <si>
-    <t>(838) 742-3423</t>
+    <t>(685) 756-4455</t>
   </si>
   <si>
-    <t>as@as.com</t>
+    <t>alagusundar.sundar@knitwellgroup.com</t>
   </si>
   <si>
-    <t>Birthday: Dec 16</t>
+    <t>Birthday: Feb 02</t>
   </si>
   <si>
     <t>********</t>

</xml_diff>

<commit_message>
Add To Cart feature added
</commit_message>
<xml_diff>
--- a/Excel/Account.xlsx
+++ b/Excel/Account.xlsx
@@ -12,21 +12,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
-    <t>new new</t>
+    <t>SFQA Test</t>
   </si>
   <si>
-    <t>(839) 758-1489</t>
+    <t>(685) 756-4455</t>
   </si>
   <si>
-    <t>new@new.com</t>
+    <t>alagusundar.sundar@knitwellgroup.com</t>
   </si>
   <si>
-    <t>Birthday: Jan 01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Subscribed to Emails</t>
+    <t>Birthday: Feb 02</t>
   </si>
   <si>
     <t>********</t>
@@ -74,7 +71,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -102,11 +99,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>5</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>